<commit_message>
Finalise les points de controle rapides IGPDE
</commit_message>
<xml_diff>
--- a/03-easy-checks/grille-audit-easy-checks.xlsx
+++ b/03-easy-checks/grille-audit-easy-checks.xlsx
@@ -220,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -310,9 +310,6 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -679,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -689,7 +686,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>IGPDE - Formation 102638 - Grille d'audit 13 Easy Checks du W3C</t>
+          <t>IGPDE - Formation 102638 - Grille d'audit 13 points de contrôle rapides du W3C</t>
         </is>
       </c>
     </row>
@@ -709,7 +706,7 @@
       <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Grille de diagnostic rapide sur les 13 Easy Checks du W3C WAI, alignée sur le RGAA 4.1.2.</t>
+          <t>Grille de diagnostic rapide sur les 13 points de contrôle rapides du W3C WAI, alignée sur le RGAA 4.1.2.</t>
         </is>
       </c>
     </row>
@@ -745,7 +742,7 @@
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Le « Taux de conformité Easy Checks » calculé ici n'est PAS le taux de conformité RGAA officiel publié en déclaration d'accessibilité.</t>
+          <t>Le « Taux de conformité points de contrôle rapides » calculé ici n'est PAS le taux de conformité RGAA officiel publié en déclaration d'accessibilité.</t>
         </is>
       </c>
     </row>
@@ -885,58 +882,58 @@
       <c r="A24" s="2" t="inlineStr"/>
       <c r="B24" s="2" t="inlineStr"/>
     </row>
-    <row r="25" ht="21" customHeight="1">
+    <row r="25" ht="26" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Règle pour l'exercice en binômes</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
+          <t>Conventions de verdict</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="26" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="B26" s="34" t="inlineStr">
-        <is>
-          <t>Les pages sont réparties entre plusieurs groupes : chaque binôme audite uniquement les pages attribuées.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Conforme - le critère est respecté sans réserve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="B27" s="34" t="inlineStr">
-        <is>
-          <t>Pour une page donnée, une seule occurrence correctement prouvée suffit à renseigner NC sur le critère ciblé.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Non conforme - un défaut objectif a été constaté.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="B28" s="34" t="inlineStr">
-        <is>
-          <t>Les autres occurrences éventuelles sont des bonus utiles pour la restitution, mais elles ne sont pas exigées pour invalider le critère.</t>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Non applicable - le critère ne s'applique pas à cette page.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="2" t="n"/>
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr"/>
     </row>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Conventions de verdict</t>
+          <t>Conventions de sévérité</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr"/>
@@ -944,124 +941,112 @@
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Bloquant</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Conforme - le critère est respecté sans réserve.</t>
+          <t>Certaines personnes sont exclues du service.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>Gênant</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Non conforme - un défaut objectif a été constaté.</t>
+          <t>Certaines personnes ont des difficultés importantes.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Mineur</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Non applicable - le critère ne s'applique pas à cette page.</t>
+          <t>L'ergonomie peut être améliorée mais l'accès reste possible.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="2" t="inlineStr"/>
-      <c r="B34" s="2" t="inlineStr"/>
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Observation à des fins d'amélioration, sans blocage.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>Conventions de sévérité</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="inlineStr"/>
       <c r="B35" s="2" t="inlineStr"/>
     </row>
     <row r="36" ht="26" customHeight="1">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>Bloquant</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Certaines personnes sont exclues du service.</t>
-        </is>
-      </c>
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Onglets du classeur</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>Gênant</t>
-        </is>
-      </c>
+      <c r="A37" s="2" t="inlineStr"/>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Certaines personnes ont des difficultés importantes.</t>
+          <t>Mode d'emploi : ce document.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>Mineur</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="inlineStr"/>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>L'ergonomie peut être améliorée mais l'accès reste possible.</t>
+          <t>Grille vierge : 13 critères à remplir pour la page auditée.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>Info</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="inlineStr"/>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Observation à des fins d'amélioration, sans blocage.</t>
+          <t>Exemple : audit illustratif sur une page type.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="26" customHeight="1">
       <c r="A40" s="2" t="inlineStr"/>
-      <c r="B40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Synthèse : décompte automatique et taux de conformité multi-pages.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="26" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>Onglets du classeur</t>
-        </is>
-      </c>
+      <c r="A41" s="2" t="inlineStr"/>
       <c r="B41" s="2" t="inlineStr"/>
     </row>
     <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="2" t="inlineStr"/>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Mode d'emploi : ce document.</t>
-        </is>
-      </c>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Références</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
     </row>
     <row r="43" ht="26" customHeight="1">
       <c r="A43" s="2" t="inlineStr"/>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Grille vierge : 13 critères à remplir pour la page auditée.</t>
+          <t>points de contrôle rapides W3C : https://www.w3.org/WAI/test-evaluate/easy-checks/</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1054,7 @@
       <c r="A44" s="2" t="inlineStr"/>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Exemple : audit illustratif sur une page type.</t>
+          <t>RGAA 4.1.2 : https://accessibilite.numerique.gouv.fr/</t>
         </is>
       </c>
     </row>
@@ -1077,43 +1062,7 @@
       <c r="A45" s="2" t="inlineStr"/>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Synthèse : décompte automatique et taux de conformité multi-pages.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr"/>
-      <c r="B46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>Références</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr"/>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>W3C Easy Checks : https://www.w3.org/WAI/test-evaluate/easy-checks/</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>RGAA 4.1.2 : https://accessibilite.numerique.gouv.fr/</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Inspiration méthodologique : grille Easy Checks de beta.gouv.fr.</t>
+          <t>Inspiration méthodologique : grille points de contrôle rapides de beta.gouv.fr.</t>
         </is>
       </c>
     </row>
@@ -1155,6 +1104,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -1163,6 +1114,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -1171,6 +1124,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -1179,6 +1134,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page de résultats de recherche</t>
@@ -1191,6 +1148,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -1199,6 +1158,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -1209,7 +1170,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -1756,7 +1717,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -1946,6 +1907,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -1954,6 +1917,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -1962,6 +1927,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -1970,6 +1937,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Document téléchargeable (PDF, DOCX, ODT)</t>
@@ -1982,6 +1951,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -1990,12 +1961,14 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Attention : les 13 Easy Checks web ne couvrent que partiellement les documents. Pour un audit formel des PDF / DOCX / ODT, utiliser PAC 2024 (outil gratuit), Acrobat Pro ou Axes4.</t>
+          <t>Attention : les 13 points de contrôle rapides web ne couvrent que partiellement les documents. Pour un audit formel des PDF / DOCX / ODT, utiliser PAC 2024 (outil gratuit), Acrobat Pro ou Axes4.</t>
         </is>
       </c>
     </row>
@@ -2007,7 +1980,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -2554,7 +2527,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -2745,6 +2718,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -2753,6 +2728,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -2761,6 +2738,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -2769,6 +2748,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page type : article, actualité ou contenu rédactionnel</t>
@@ -2781,6 +2762,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -2789,6 +2772,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -2799,7 +2784,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -3346,7 +3331,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -3536,6 +3521,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -3544,6 +3531,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -3552,6 +3541,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -3560,6 +3551,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page type : formulaire de démarche ou saisie multi-étape</t>
@@ -3572,6 +3565,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -3580,6 +3575,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -3590,7 +3587,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -4137,7 +4134,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -4327,6 +4324,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -4335,6 +4334,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -4343,6 +4344,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -4351,6 +4354,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page type : liste / rubrique / résultats de navigation</t>
@@ -4363,6 +4368,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -4371,6 +4378,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -4381,7 +4390,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -4928,7 +4937,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -5118,6 +5127,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Dupont Jean</t>
@@ -5130,6 +5141,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>4 juin 2026</t>
@@ -5142,6 +5155,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>https://exemple.gouv.fr/accueil</t>
@@ -5154,6 +5169,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page d'accueil ministère</t>
@@ -5166,6 +5183,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Firefox 122 sous Windows 11</t>
@@ -5178,6 +5197,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
           <t>HeadingsMap, DevTools, NVDA</t>
@@ -5192,7 +5213,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -5927,7 +5948,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -6154,7 +6175,7 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
     </row>
@@ -6828,7 +6849,7 @@
       <c r="D17" s="10" t="inlineStr"/>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Au moins un document représentatif. Attention : les 13 Easy Checks web ne couvrent qu'en partie les documents. Pour un audit complet, utiliser PAC 2024 (gratuit), Acrobat Pro ou Axes4.</t>
+          <t>Au moins un document représentatif. Attention : les 13 points de contrôle rapides web ne couvrent qu'en partie les documents. Pour un audit complet, utiliser PAC 2024 (gratuit), Acrobat Pro ou Axes4.</t>
         </is>
       </c>
     </row>
@@ -6983,6 +7004,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -6991,6 +7014,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -6999,6 +7024,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -7007,6 +7034,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page d'accueil</t>
@@ -7019,6 +7048,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -7027,6 +7058,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -7037,7 +7070,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -7584,7 +7617,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -7774,6 +7807,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -7782,6 +7817,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -7790,6 +7827,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -7798,6 +7837,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page « Mentions légales »</t>
@@ -7810,6 +7851,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -7818,6 +7861,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -7828,7 +7873,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -8375,7 +8420,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -8565,6 +8610,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -8573,6 +8620,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -8581,6 +8630,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -8589,6 +8640,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Déclaration d'accessibilité</t>
@@ -8601,6 +8654,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -8609,6 +8664,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -8619,7 +8676,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -9166,7 +9223,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -9356,6 +9413,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -9364,6 +9423,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -9372,6 +9433,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -9380,6 +9443,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page « Plan du site »</t>
@@ -9392,6 +9457,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -9400,6 +9467,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -9410,7 +9479,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -9957,7 +10026,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -10147,6 +10216,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -10155,6 +10226,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -10163,6 +10236,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -10171,6 +10246,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page « Contact »</t>
@@ -10183,6 +10260,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -10191,6 +10270,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -10201,7 +10282,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -10748,7 +10829,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -10938,6 +11019,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -10946,6 +11029,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -10954,6 +11039,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -10962,6 +11049,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page « Aide » / FAQ</t>
@@ -10974,6 +11063,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -10982,6 +11073,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -10992,7 +11085,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -11539,7 +11632,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">
@@ -11729,6 +11822,8 @@
           <t>Auditeur / auditrice</t>
         </is>
       </c>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
       <c r="D1" s="2" t="inlineStr"/>
     </row>
     <row r="2" ht="26" customHeight="1">
@@ -11737,6 +11832,8 @@
           <t>Date de l'audit</t>
         </is>
       </c>
+      <c r="B2" s="19" t="n"/>
+      <c r="C2" s="19" t="n"/>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="26" customHeight="1">
@@ -11745,6 +11842,8 @@
           <t>URL de la page auditée</t>
         </is>
       </c>
+      <c r="B3" s="19" t="n"/>
+      <c r="C3" s="19" t="n"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
@@ -11753,6 +11852,8 @@
           <t>Intitulé de la page</t>
         </is>
       </c>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Page d'authentification / connexion</t>
@@ -11765,6 +11866,8 @@
           <t>Navigateur et version</t>
         </is>
       </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
       <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
@@ -11773,6 +11876,8 @@
           <t>Outils utilisés</t>
         </is>
       </c>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
       <c r="D6" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
@@ -11783,7 +11888,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Easy Check</t>
+          <t>Point de contrôle rapide</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -12330,7 +12435,7 @@
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Taux de conformité Easy Checks</t>
+          <t>Taux de conformité points de contrôle rapides</t>
         </is>
       </c>
       <c r="F28" s="21">

</xml_diff>

<commit_message>
Qualité : aligner le pack IGPDE et ses contrôles
Changelog: non applicable — corrections internes de cohérence et de contrôle du pack.

Backlog: non applicable — suivi actualisé dans le PRD, le ticket T16 et la todo.
</commit_message>
<xml_diff>
--- a/03-easy-checks/grille-audit-easy-checks.xlsx
+++ b/03-easy-checks/grille-audit-easy-checks.xlsx
@@ -7516,7 +7516,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>53-55</t>
+          <t>84-86</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>87</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -7612,7 +7612,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>57-58</t>
+          <t>88-89</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -7660,7 +7660,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>59-60</t>
+          <t>90-91</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -7708,7 +7708,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>92</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -7756,7 +7756,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>62-65</t>
+          <t>93-96</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -7804,7 +7804,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>97</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -7852,7 +7852,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>98</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -7900,7 +7900,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>68-69</t>
+          <t>99-100</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -7948,7 +7948,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>101</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -7996,7 +7996,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>102</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>72-74</t>
+          <t>105-107</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>108</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">

</xml_diff>

<commit_message>
feat(web): ajout du test d'espacement
</commit_message>
<xml_diff>
--- a/03-easy-checks/grille-audit-easy-checks.xlsx
+++ b/03-easy-checks/grille-audit-easy-checks.xlsx
@@ -4192,7 +4192,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>À 200 % et dans une fenêtre étroite, les contenus restent-ils lisibles et utilisables sans perte d'information ?</t>
+          <t>À 200 %, dans une fenêtre étroite et avec un espacement du texte renforcé, les contenus restent-ils lisibles et utilisables sans perte d'information ?</t>
         </is>
       </c>
     </row>
@@ -4204,7 +4204,7 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>1.4.4 - Redimensionnement du texte ; 1.4.10 - Redistribution</t>
+          <t>1.4.4 - Redimensionnement du texte ; 1.4.10 - Redistribution ; 1.4.12 - Espacement du texte</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>10.4, 10.11</t>
+          <t>10.4, 10.11, 10.12</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Zoomer à 200 %, puis tester séparément une zone d'affichage de 320 CSS px et parcourir tout le contenu.</t>
+          <t>Zoomer à 200 %, puis tester séparément une zone d'affichage de 320 CSS px. Activer ensuite le bookmarklet « 10.12 Espacement » et parcourir tout le contenu.</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Aucun texte coupé ou superposé. Contenus et commandes utilisables. Pas de défilement dans deux directions pour lire le contenu courant.</t>
+          <t>Aucun texte coupé ou superposé. Contenus et commandes utilisables. Pas de défilement dans deux directions pour lire le contenu courant. Aucun contenu perdu après modification de l'espacement du texte.</t>
         </is>
       </c>
     </row>

</xml_diff>